<commit_message>
Rebuild leaked customer-toggle widget as interactive quicklinks-toggle block
The '.homepagewishlistcomp' persona bar on tataaia.com (a 'new customer /
existing customer' toggle with an action dropdown) was flattened into loose
paragraphs, lists and stray icons inside the Top Selling Plans section.
Rebuild it as a proper interactive block:
- blocks/quicklinks-toggle: container + repeating item (label + prompt/links);
  JS renders a persona toggle + action select + red go-arrow, switching the
  option list and prompt per persona; CSS matches the live pill/toggle styling
- parser + bundle: extract both personas (new -> 'I want to', existing ->
  'Help me to') from .homepagewishlistcomp into two rows
- page-templates + bundle: new s2b section mapping .homepagewishlistcomp
- reimported (2 personas, 10 links) and regenerated JCR (19 sections, validates)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-home.report.xlsx
+++ b/tools/importer/reports/import-home.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero-promo","hero-banner","cards-plan","cards-persona","cards-quicklink","cards-promo","cards-award","cards-stats","carousel-banner","cards-article","columns-panels","columns-panels","columns-panels","accordion-list","accordion-list","accordion-list","accordion-list","accordion-list","carousel-review","carousel-video","quote-callout","table-data","tabs-links","tabs-links","form","form"]</t>
+    <t>["hero-promo","hero-banner","cards-plan","quicklinks-toggle","cards-persona","cards-quicklink","cards-promo","cards-award","cards-stats","carousel-banner","cards-article","columns-panels","columns-panels","columns-panels","accordion-list","accordion-list","accordion-list","accordion-list","accordion-list","carousel-review","carousel-video","quote-callout","table-data","tabs-links","tabs-links","form","form"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-09-16T12:10:06.891Z</t>
+    <t>2026-09-16T12:21:17.144Z</t>
   </si>
   <si>
     <t>Life Insurance - Best Life Insurance Online in India 2026</t>

</xml_diff>

<commit_message>
Restore 'Looking to buy a new life insurance plan?' call-back form section
The .tte-form-redesign section (heading 'Looking to buy a new life insurance
plan?' + a call-back form) was mapped to the same JSON as the 'Know more…2
steps' calc form, so it rendered without its own heading/fields. Give it a
dedicated EDS form:
- content/looking-to-buy-callback.json: heading + 'Our experts are happy to
  help you!' subtext, NRI Yes/No, Name, Mobile (+91), Plan, consent, 'Get a
  Call Back' submit
- map .tte-form-redesign -> looking-to-buy-callback.json in the form parser +
  bundle FORM_DEFINITIONS/FORM_ACTIONS
- gate the tabbed plan-picker layout to the calc form only (has dateOfBirth);
  the call-back form stays a plain vertical form
- reimported (2 distinct forms) and regenerated JCR (validates)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-home.report.xlsx
+++ b/tools/importer/reports/import-home.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero-promo","hero-banner","cards-plan","quicklinks-toggle","columns-product-recom","cards-persona","cards-quicklink","cards-promo","cards-award","cards-stats","carousel-banner","cards-article","columns-panels","columns-panels","columns-panels","accordion-list","accordion-list","accordion-list","accordion-list","accordion-list","carousel-review","carousel-video","quote-callout","table-data","tabs-links","tabs-links","form","form"]</t>
+    <t>["hero-promo","hero-banner","cards-plan","quicklinks-toggle","columns-product-recom","cards-persona","cards-quicklink","cards-promo","cards-award","cards-stats","carousel-banner","cards-article","columns-panels","columns-panels","columns-panels","accordion-list","accordion-list","accordion-list","accordion-list","accordion-list","carousel-review","carousel-video","table-data","tabs-links","tabs-links","form","form"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-09-16T13:01:39.346Z</t>
+    <t>2026-09-16T17:02:34.798Z</t>
   </si>
   <si>
     <t>Life Insurance - Best Life Insurance Online in India 2026</t>

</xml_diff>